<commit_message>
Sync 2026-09-02: 10 Katana status updates + 23 new tasks (#524-#546)
Status changes: #305,#319 Done; #320,#323,#325,#336,#338,#340,#364 In review; #345 Backlog
New tasks: ABI.Unity issues #1107-#1129 (General UI/UX, Recipe, Robot Control, Safety, Settings Panel, Layer Panel, Scaling)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016CmAfMJ97kwanzK1vWp6P5
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A1CB4B-2609-4B1E-B10C-A14C0AE29F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5DA5E2-D206-4C0C-9B1D-1F5613E5A13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2962" uniqueCount="1086">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3121" uniqueCount="1134">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -3295,6 +3295,150 @@
   </si>
   <si>
     <t>Beckoff IPC reaches &gt;4 GHz speed; tested with phantom mode and production mode, IPC performs well.</t>
+  </si>
+  <si>
+    <t>When you expand the entire window, hide the task bar.</t>
+  </si>
+  <si>
+    <t>When the user expands the entire window, hide the task bar.</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>[2026-08-18]</t>
+  </si>
+  <si>
+    <t>Permission lock: default values must remain accessible to all default users.</t>
+  </si>
+  <si>
+    <t>Permission lock: default values must remain accessible. If allowed range starts at 1, change default to 1 for all users.</t>
+  </si>
+  <si>
+    <t>Avoid showing Contact ABI for range validation as much as possible.</t>
+  </si>
+  <si>
+    <t>For Khurram to follow up. [2026-08-18]</t>
+  </si>
+  <si>
+    <t>Only Admins and Super Admins can change custom distribution.</t>
+  </si>
+  <si>
+    <t>Only Admins and Super Admins can change custom distribution; all other users see default distribution.</t>
+  </si>
+  <si>
+    <t>Make sure the Start and Stop buttons are the same size on the home screen.</t>
+  </si>
+  <si>
+    <t>Hide Recipe Comparison from all users except Super Admins.</t>
+  </si>
+  <si>
+    <t>Hide Recipe Comparison from all users except Super Admins (not fully tested). Clarify cutstyle meaning.</t>
+  </si>
+  <si>
+    <t>When the tool-change flag is enabled, enable tool selection for all users.</t>
+  </si>
+  <si>
+    <t>When tool-change flag is enabled, enable tool selection for all users. Overall check for Recipe Add/Edit bugs.</t>
+  </si>
+  <si>
+    <t>bug, Feature</t>
+  </si>
+  <si>
+    <t>Potential overlap with existing tool-selection task. [2026-08-18]</t>
+  </si>
+  <si>
+    <t>Add a loading spinner for recipes.</t>
+  </si>
+  <si>
+    <t>Fix Edit Recipe pages so they do not use a scrollable page.</t>
+  </si>
+  <si>
+    <t>Potential overlap with existing scrollbar task. [2026-08-18]</t>
+  </si>
+  <si>
+    <t>When cloning a recipe, show a popup that allows the user to rename the cloned recipe.</t>
+  </si>
+  <si>
+    <t>Add Group Control, Batch Control, and All Robots control options.</t>
+  </si>
+  <si>
+    <t>Fix the Last Image page layout.</t>
+  </si>
+  <si>
+    <t>Remove scrolling, retain pagination, fix first image popup not opening after moving to next page.</t>
+  </si>
+  <si>
+    <t>Allow reports to be deleted.</t>
+  </si>
+  <si>
+    <t>PLC Emergency error not shown in Katana when door is opened.</t>
+  </si>
+  <si>
+    <t>Opened the door while PLC was in Emergency error; Katana was not showing any error.</t>
+  </si>
+  <si>
+    <t>DG noticed this on the cell. [2026-08-20]</t>
+  </si>
+  <si>
+    <t>Calibration offset page: table header overlays the settings menu when opened.</t>
+  </si>
+  <si>
+    <t>On the calibration offset page, opening the left settings menu causes the table header to overlay the settings menu.</t>
+  </si>
+  <si>
+    <t>[2026-08-20]</t>
+  </si>
+  <si>
+    <t>Fix robot labels offset; travel direction angle is 180 degrees wrong.</t>
+  </si>
+  <si>
+    <t>Fix the robot labels offset to top; travel direction angle is wrong - 180 degrees opposite.</t>
+  </si>
+  <si>
+    <t>Changing custom distribution causes settings panel to jump from 2 to 4 pages.</t>
+  </si>
+  <si>
+    <t>Changing the custom distribution in the settings panel causes the advanced tab to increase from 2 to 4 pages.</t>
+  </si>
+  <si>
+    <t>Layer panel: Robot IDs and Distribution columns should be swapped.</t>
+  </si>
+  <si>
+    <t>Robot ID column shows distribution limits and distribution column shows robot IDs - they should be swapped.</t>
+  </si>
+  <si>
+    <t>Settings panel is unstable and glitchy - value changes affect items and pagination.</t>
+  </si>
+  <si>
+    <t>Settings panel is not stable and glitchy; a value change causes items and pagination to change unexpectedly.</t>
+  </si>
+  <si>
+    <t>Scaling Y should be inverted.</t>
+  </si>
+  <si>
+    <t>Page freezes during phantom mode; stuck again after navigating to calibration offsets.</t>
+  </si>
+  <si>
+    <t>Page froze while phantom mode was running. After refresh it worked, then got stuck again after navigating to calibration offsets.</t>
+  </si>
+  <si>
+    <t>Stop button should trigger cycle stop, not immediate stop.</t>
+  </si>
+  <si>
+    <t>Stop button should be cycle stop, not immediate stop.</t>
+  </si>
+  <si>
+    <t>Triggers cycle stop same as WPF, check with Khurram. [2026-08-27]</t>
+  </si>
+  <si>
+    <t>Cycle stop button on each robot stays disabled after starting.</t>
+  </si>
+  <si>
+    <t>Cycle stop button on each robot is disabled when starting and continues to stay disabled/locked.</t>
+  </si>
+  <si>
+    <t>[2026-08-27]</t>
   </si>
 </sst>
 </file>
@@ -5176,7 +5320,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1054"/>
+  <dimension ref="A1:N1077"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -12939,7 +13083,7 @@
         <v>594</v>
       </c>
       <c r="E288" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F288" t="s">
         <v>431</v>
@@ -13318,7 +13462,7 @@
         <v>66</v>
       </c>
       <c r="E302" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F302" t="s">
         <v>428</v>
@@ -13343,7 +13487,7 @@
         <v>609</v>
       </c>
       <c r="E303" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F303" t="s">
         <v>428</v>
@@ -13418,7 +13562,7 @@
         <v>66</v>
       </c>
       <c r="E306" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F306" t="s">
         <v>431</v>
@@ -13468,7 +13612,7 @@
         <v>614</v>
       </c>
       <c r="E308" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F308" t="s">
         <v>428</v>
@@ -13763,7 +13907,7 @@
         <v>625</v>
       </c>
       <c r="E319" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F319" t="s">
         <v>428</v>
@@ -13816,7 +13960,7 @@
         <v>61</v>
       </c>
       <c r="E321" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F321" t="s">
         <v>431</v>
@@ -13877,7 +14021,7 @@
         <v>61</v>
       </c>
       <c r="E323" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F323" t="s">
         <v>428</v>
@@ -14002,7 +14146,7 @@
         <v>61</v>
       </c>
       <c r="E328" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F328" t="s">
         <v>431</v>
@@ -14482,7 +14626,7 @@
         <v>66</v>
       </c>
       <c r="E347" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F347" t="s">
         <v>431</v>
@@ -20978,6 +21122,598 @@
         <v>1085</v>
       </c>
       <c r="M1054" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1055">
+        <v>524</v>
+      </c>
+      <c r="B1055" s="3" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C1055" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E1055" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1055" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1055" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1055" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1055" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1056">
+        <v>525</v>
+      </c>
+      <c r="B1056" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C1056" s="3" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E1056" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1056" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1056" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1056" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1056" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1057">
+        <v>526</v>
+      </c>
+      <c r="B1057" s="3" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C1057" s="3" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E1057" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1057" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1057" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1057" t="s">
+        <v>1093</v>
+      </c>
+      <c r="M1057" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1058">
+        <v>527</v>
+      </c>
+      <c r="B1058" s="3" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C1058" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E1058" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1058" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1058" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1058" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1058" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1059">
+        <v>528</v>
+      </c>
+      <c r="B1059" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C1059" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E1059" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1059" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1059" t="s">
+        <v>874</v>
+      </c>
+      <c r="L1059" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1059" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1060">
+        <v>529</v>
+      </c>
+      <c r="B1060" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C1060" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E1060" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1060" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1060" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1060" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1060" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1061">
+        <v>530</v>
+      </c>
+      <c r="B1061" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C1061" s="3" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1061" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1061" t="s">
+        <v>1101</v>
+      </c>
+      <c r="L1061" t="s">
+        <v>1102</v>
+      </c>
+      <c r="M1061" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1062">
+        <v>531</v>
+      </c>
+      <c r="B1062" s="3" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C1062" s="3" t="s">
+        <v>1103</v>
+      </c>
+      <c r="E1062" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1062" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1062" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1062" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1062" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1063">
+        <v>532</v>
+      </c>
+      <c r="B1063" s="3" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C1063" s="3" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E1063" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1063" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1063" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1063" t="s">
+        <v>1105</v>
+      </c>
+      <c r="M1063" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1064">
+        <v>533</v>
+      </c>
+      <c r="B1064" s="3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C1064" s="3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="E1064" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1064" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1064" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1064" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1064" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1065">
+        <v>534</v>
+      </c>
+      <c r="B1065" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C1065" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E1065" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1065" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1065" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1065" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1065" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1066">
+        <v>535</v>
+      </c>
+      <c r="B1066" s="3" t="s">
+        <v>1108</v>
+      </c>
+      <c r="C1066" s="3" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E1066" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1066" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1066" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1066" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1066" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1067">
+        <v>536</v>
+      </c>
+      <c r="B1067" s="3" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C1067" s="3" t="s">
+        <v>1110</v>
+      </c>
+      <c r="E1067" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1067" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1067" t="s">
+        <v>1088</v>
+      </c>
+      <c r="L1067" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M1067" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1068">
+        <v>537</v>
+      </c>
+      <c r="B1068" s="3" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C1068" s="3" t="s">
+        <v>1112</v>
+      </c>
+      <c r="E1068" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1068" t="s">
+        <v>427</v>
+      </c>
+      <c r="K1068" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1068" t="s">
+        <v>1113</v>
+      </c>
+      <c r="M1068" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1069">
+        <v>538</v>
+      </c>
+      <c r="B1069" s="3" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C1069" s="3" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E1069" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1069" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1069" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1069" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1069" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1070">
+        <v>539</v>
+      </c>
+      <c r="B1070" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C1070" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="E1070" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1070" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1070" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1070" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1070" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1071">
+        <v>540</v>
+      </c>
+      <c r="B1071" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C1071" s="3" t="s">
+        <v>1120</v>
+      </c>
+      <c r="E1071" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1071" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1071" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1071" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1071" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1072">
+        <v>541</v>
+      </c>
+      <c r="B1072" s="3" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C1072" s="3" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E1072" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1072" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1072" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1072" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1072" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1073">
+        <v>542</v>
+      </c>
+      <c r="B1073" s="3" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C1073" s="3" t="s">
+        <v>1124</v>
+      </c>
+      <c r="E1073" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1073" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1073" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1073" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1073" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1074">
+        <v>543</v>
+      </c>
+      <c r="B1074" s="3" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C1074" s="3" t="s">
+        <v>1125</v>
+      </c>
+      <c r="E1074" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1074" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1074" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1074" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1074" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1075">
+        <v>544</v>
+      </c>
+      <c r="B1075" s="3" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C1075" s="3" t="s">
+        <v>1127</v>
+      </c>
+      <c r="E1075" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1075" t="s">
+        <v>431</v>
+      </c>
+      <c r="K1075" t="s">
+        <v>717</v>
+      </c>
+      <c r="L1075" t="s">
+        <v>1116</v>
+      </c>
+      <c r="M1075" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1076">
+        <v>545</v>
+      </c>
+      <c r="B1076" s="3" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C1076" s="3" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E1076" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1076" t="s">
+        <v>431</v>
+      </c>
+      <c r="L1076" t="s">
+        <v>1130</v>
+      </c>
+      <c r="M1076" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1077">
+        <v>546</v>
+      </c>
+      <c r="B1077" s="3" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C1077" s="3" t="s">
+        <v>1132</v>
+      </c>
+      <c r="E1077" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1077" t="s">
+        <v>431</v>
+      </c>
+      <c r="L1077" t="s">
+        <v>1133</v>
+      </c>
+      <c r="M1077" t="s">
         <v>69</v>
       </c>
     </row>
@@ -21107,6 +21843,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -21361,15 +22106,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -21382,6 +22118,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21400,14 +22144,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add 74 Eye-Q + AI_CORE Sodebo tasks (#547-#620): ABI.Unity issues #1130-#1203
Scope: Eye-Q | Assignee: MauricioDuqueABI
GitHub issues #1130-#1203 created in ABI.Unity, added to KII project with
Status (Done/In progress/Backlog), Scope=Eye-Q, and Estimate field set.
Monday.com subitems created under Eye-Q parent (board 18394803683).
task_mapping.json: 546->620 entries. project_data.json: 527->601 tasks.
project_time_sheet.xlsx: rows 1078-1151 added (KII Tasks sheet).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016CmAfMJ97kwanzK1vWp6P5
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5DA5E2-D206-4C0C-9B1D-1F5613E5A13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497D3D87-B10F-49BA-A317-4A6C351579D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3121" uniqueCount="1134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3565" uniqueCount="1283">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -3439,6 +3439,453 @@
   </si>
   <si>
     <t>[2026-08-27]</t>
+  </si>
+  <si>
+    <t>AI/RAW image separation: display annotated inference image in AI pane and original in RAW pane</t>
+  </si>
+  <si>
+    <t>Display annotated inference image in AI pane and original image in RAW pane.</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Scan-result ingestion: configure EyeQ to receive AI_CORE results through /api/ingest/scan-result</t>
+  </si>
+  <si>
+    <t>Configure EyeQ to receive AI_CORE results through /api/ingest/scan-result.</t>
+  </si>
+  <si>
+    <t>Missing height handling: allow width and length to be stored when height cannot be measured</t>
+  </si>
+  <si>
+    <t>Allow width and length to be stored when height cannot be measured.</t>
+  </si>
+  <si>
+    <t>Database scan storage: store AI_CORE scan results, products and measurements in PostgreSQL</t>
+  </si>
+  <si>
+    <t>Store AI_CORE scan results, products and measurements in PostgreSQL.</t>
+  </si>
+  <si>
+    <t>Trends integration: display product measurements, counts and recent images</t>
+  </si>
+  <si>
+    <t>Display product measurements, counts and recent images.</t>
+  </si>
+  <si>
+    <t>CSV measurement export: export stored product and recipe information</t>
+  </si>
+  <si>
+    <t>Export stored product and recipe information.</t>
+  </si>
+  <si>
+    <t>Duplicate scan investigation: investigate inflated boards and product counts</t>
+  </si>
+  <si>
+    <t>Investigate inflated boards and product counts.</t>
+  </si>
+  <si>
+    <t>PostgreSQL development setup: install/configure PostgreSQL and create EyeQ database for development</t>
+  </si>
+  <si>
+    <t>Install/configure PostgreSQL and create EyeQ database for development.</t>
+  </si>
+  <si>
+    <t>PostgreSQL port conflict: avoid conflict with an existing PostgreSQL 18 instance on port 5432</t>
+  </si>
+  <si>
+    <t>Avoid conflict with an existing PostgreSQL 18 instance on port 5432.</t>
+  </si>
+  <si>
+    <t>Database provisioner: bundle database creation and migration with the installer</t>
+  </si>
+  <si>
+    <t>Bundle database creation and migration with the installer.</t>
+  </si>
+  <si>
+    <t>AI_CORE service installation: package AI_CORE as a Windows service alongside EyeQ</t>
+  </si>
+  <si>
+    <t>Package AI_CORE as a Windows service alongside EyeQ.</t>
+  </si>
+  <si>
+    <t>AI_CORE writable data path: move .agent-data and runtime state outside Program Files</t>
+  </si>
+  <si>
+    <t>Move .agent-data and runtime state outside Program Files.</t>
+  </si>
+  <si>
+    <t>EyeQ Windows service: install EyeQ as an automatically starting service</t>
+  </si>
+  <si>
+    <t>Install EyeQ as an automatically starting service.</t>
+  </si>
+  <si>
+    <t>Recovery supervisor: add monitoring and automatic service recovery</t>
+  </si>
+  <si>
+    <t>Add monitoring and automatic service recovery.</t>
+  </si>
+  <si>
+    <t>EyeQ launcher: add desktop launcher for EyeQ and AI_CORE</t>
+  </si>
+  <si>
+    <t>Add desktop launcher for EyeQ and AI_CORE.</t>
+  </si>
+  <si>
+    <t>Launcher icon: add EyeQ icon to installed shortcut</t>
+  </si>
+  <si>
+    <t>Add EyeQ icon to installed shortcut.</t>
+  </si>
+  <si>
+    <t>Offline all-in-one installer: build installer containing EyeQ, AI_CORE and PostgreSQL</t>
+  </si>
+  <si>
+    <t>Build installer containing EyeQ, AI_CORE and PostgreSQL.</t>
+  </si>
+  <si>
+    <t>Clean uninstaller: provide removal of installed services and applications</t>
+  </si>
+  <si>
+    <t>Provide removal of installed services and applications.</t>
+  </si>
+  <si>
+    <t>Copy-and-run fallback: document manual folder-copy deployment</t>
+  </si>
+  <si>
+    <t>Document manual folder-copy deployment.</t>
+  </si>
+  <si>
+    <t>Installer documentation: write installation, update and recovery instructions in Obsidian</t>
+  </si>
+  <si>
+    <t>Write installation, update and recovery instructions in Obsidian.</t>
+  </si>
+  <si>
+    <t>Firewall access: allow external access to EyeQ on TCP port 5000</t>
+  </si>
+  <si>
+    <t>Allow external access to EyeQ on TCP port 5000.</t>
+  </si>
+  <si>
+    <t>Bind EyeQ externally: ensure EyeQ listens on all network interfaces</t>
+  </si>
+  <si>
+    <t>Ensure EyeQ listens on all network interfaces.</t>
+  </si>
+  <si>
+    <t>Tablet access diagnosis: diagnose why AI_CORE was reachable but EyeQ was not</t>
+  </si>
+  <si>
+    <t>Diagnose why AI_CORE was reachable but EyeQ was not.</t>
+  </si>
+  <si>
+    <t>API-key packaging: ensure packaged AI_CORE and EyeQ share an ingest API key</t>
+  </si>
+  <si>
+    <t>Ensure packaged AI_CORE and EyeQ share an ingest API key.</t>
+  </si>
+  <si>
+    <t>Client file selection: preserve browser-side image and video upload</t>
+  </si>
+  <si>
+    <t>Preserve browser-side image and video upload.</t>
+  </si>
+  <si>
+    <t>Server file selection: add server-side file browsing option</t>
+  </si>
+  <si>
+    <t>Add server-side file browsing option.</t>
+  </si>
+  <si>
+    <t>Missing Tkinter failure: remove reliance on Tkinter for packaged file browsing</t>
+  </si>
+  <si>
+    <t>Remove reliance on Tkinter for packaged file browsing.</t>
+  </si>
+  <si>
+    <t>RealSense camera deployment: diagnose RealSense discovery after installation</t>
+  </si>
+  <si>
+    <t>Diagnose RealSense discovery after installation.</t>
+  </si>
+  <si>
+    <t>Camera-network discovery: make RealSense detection independent of adapter name</t>
+  </si>
+  <si>
+    <t>Make RealSense detection independent of adapter name.</t>
+  </si>
+  <si>
+    <t>Jumbo packet configuration: configure compatible Ethernet jumbo frames</t>
+  </si>
+  <si>
+    <t>Configure compatible Ethernet jumbo frames.</t>
+  </si>
+  <si>
+    <t>Camera calibration source: allow 2D Metrology to consume saved camera calibration</t>
+  </si>
+  <si>
+    <t>Allow 2D Metrology to consume saved camera calibration.</t>
+  </si>
+  <si>
+    <t>Calibration discrepancy: fix displayed manual value remaining at 7.46 px/mm</t>
+  </si>
+  <si>
+    <t>Fix displayed manual value remaining at 7.46 px/mm.</t>
+  </si>
+  <si>
+    <t>Manual metrology UI: hide camera selector when manual pixels/mm is selected</t>
+  </si>
+  <si>
+    <t>Hide camera selector when manual pixels/mm is selected.</t>
+  </si>
+  <si>
+    <t>Recipe detector integration: receive AI-detected recipe information from AI_CORE</t>
+  </si>
+  <si>
+    <t>Receive AI-detected recipe information from AI_CORE.</t>
+  </si>
+  <si>
+    <t>AI recipe fields: store recipe detected by AI and its decision metadata</t>
+  </si>
+  <si>
+    <t>Store recipe detected by AI and its decision metadata.</t>
+  </si>
+  <si>
+    <t>Optional recipe input: allow publisher to operate when recipe detector port is disconnected</t>
+  </si>
+  <si>
+    <t>Allow publisher to operate when recipe detector port is disconnected.</t>
+  </si>
+  <si>
+    <t>Recipe-source policy: keep EyeQ as authoritative recipe source with optional AI recommendation</t>
+  </si>
+  <si>
+    <t>Keep EyeQ as authoritative recipe source with optional AI recommendation.</t>
+  </si>
+  <si>
+    <t>Recipe selection mode: document how to change recipe selection from PLC to manual</t>
+  </si>
+  <si>
+    <t>Document how to change recipe selection from PLC to manual.</t>
+  </si>
+  <si>
+    <t>AI view feature flags: diagnose missing AI/side-by-side controls</t>
+  </si>
+  <si>
+    <t>Diagnose missing AI/side-by-side controls.</t>
+  </si>
+  <si>
+    <t>PostgreSQL feature query: diagnose incorrect FeatureSettings SQL query</t>
+  </si>
+  <si>
+    <t>Diagnose incorrect FeatureSettings SQL query.</t>
+  </si>
+  <si>
+    <t>Recipes-page load reduction: remove expensive header calculation from /recipes</t>
+  </si>
+  <si>
+    <t>Remove expensive header calculation from /recipes.</t>
+  </si>
+  <si>
+    <t>Reviewer critical fixes: review 24 reported EyeQ issues and propose corrections</t>
+  </si>
+  <si>
+    <t>Review 24 reported EyeQ issues and propose corrections.</t>
+  </si>
+  <si>
+    <t>Scan-source statistics: restore 3D-only production-stat semantics</t>
+  </si>
+  <si>
+    <t>Restore 3D-only production-stat semantics.</t>
+  </si>
+  <si>
+    <t>Hardcoded ingest self-call: replace/plan removal of hardcoded localhost self-HTTP call</t>
+  </si>
+  <si>
+    <t>Replace/plan removal of hardcoded localhost self-HTTP call.</t>
+  </si>
+  <si>
+    <t>CSV injection protection: escape and quote AI recipe fields in CSV</t>
+  </si>
+  <si>
+    <t>Escape and quote AI recipe fields in CSV.</t>
+  </si>
+  <si>
+    <t>Machine ID attribution: remove hardcoded machine ID assumptions</t>
+  </si>
+  <si>
+    <t>Remove hardcoded machine ID assumptions.</t>
+  </si>
+  <si>
+    <t>Image retention risk: identify unbounded AI preview storage</t>
+  </si>
+  <si>
+    <t>Identify unbounded AI preview storage.</t>
+  </si>
+  <si>
+    <t>Ingest concurrency: identify process-wide serialization and missing distributed uniqueness</t>
+  </si>
+  <si>
+    <t>Identify process-wide serialization and missing distributed uniqueness.</t>
+  </si>
+  <si>
+    <t>EyeQ localization: synchronize EyeQ language with AI_CORE</t>
+  </si>
+  <si>
+    <t>Synchronize EyeQ language with AI_CORE.</t>
+  </si>
+  <si>
+    <t>Access-level model: implement Levels 0-4 while preserving legacy roles</t>
+  </si>
+  <si>
+    <t>Implement Levels 0-4 while preserving legacy roles.</t>
+  </si>
+  <si>
+    <t>Anonymous live access: allow logged-out users to view live data and charts</t>
+  </si>
+  <si>
+    <t>Allow logged-out users to view live data and charts.</t>
+  </si>
+  <si>
+    <t>Operator permissions: permit operators to load recipes</t>
+  </si>
+  <si>
+    <t>Permit operators to load recipes.</t>
+  </si>
+  <si>
+    <t>Supervisor permissions: permit supervisors to load and create recipes</t>
+  </si>
+  <si>
+    <t>Permit supervisors to load and create recipes.</t>
+  </si>
+  <si>
+    <t>DataViewer permissions: permit collected-data viewing and CSV download</t>
+  </si>
+  <si>
+    <t>Permit collected-data viewing and CSV download.</t>
+  </si>
+  <si>
+    <t>Admin permissions: permit recipe management, users and configuration</t>
+  </si>
+  <si>
+    <t>Permit recipe management, users and configuration.</t>
+  </si>
+  <si>
+    <t>Tech permissions: restrict Tech to routine camera/backup maintenance</t>
+  </si>
+  <si>
+    <t>Restrict Tech to routine camera/backup maintenance.</t>
+  </si>
+  <si>
+    <t>User account management: add Operator, Supervisor and DataViewer role choices</t>
+  </si>
+  <si>
+    <t>Add Operator, Supervisor and DataViewer role choices.</t>
+  </si>
+  <si>
+    <t>Access matrix: add capability-versus-role table to /UserAccounts</t>
+  </si>
+  <si>
+    <t>Add capability-versus-role table to /UserAccounts.</t>
+  </si>
+  <si>
+    <t>Remove Level 0 account creation: prevent creation of Level 0/User accounts</t>
+  </si>
+  <si>
+    <t>Prevent creation of Level 0/User accounts.</t>
+  </si>
+  <si>
+    <t>Password entry protection: require passwords and discourage browser credential storage</t>
+  </si>
+  <si>
+    <t>Require passwords and discourage browser credential storage.</t>
+  </si>
+  <si>
+    <t>EyeQ missing styles: diagnose oversized icons and missing component styling</t>
+  </si>
+  <si>
+    <t>Diagnose oversized icons and missing component styling.</t>
+  </si>
+  <si>
+    <t>Production-style local launch: launch EyeQ from published output to serve all static assets</t>
+  </si>
+  <si>
+    <t>Launch EyeQ from published output to serve all static assets.</t>
+  </si>
+  <si>
+    <t>Blank chart panels: fix ApexCharts localization lifecycle exception</t>
+  </si>
+  <si>
+    <t>Fix ApexCharts localization lifecycle exception.</t>
+  </si>
+  <si>
+    <t>Height chart overflow: make Height Profile chart responsive to viewport height</t>
+  </si>
+  <si>
+    <t>Make Height Profile chart responsive to viewport height.</t>
+  </si>
+  <si>
+    <t>Recipe statistics table: add independent daily Stats table</t>
+  </si>
+  <si>
+    <t>Add independent daily Stats table.</t>
+  </si>
+  <si>
+    <t>Statistics backfill: populate Stats from historical scans</t>
+  </si>
+  <si>
+    <t>Populate Stats from historical scans.</t>
+  </si>
+  <si>
+    <t>Atomic statistics updates: update daily counters as scans are stored</t>
+  </si>
+  <si>
+    <t>Update daily counters as scans are stored.</t>
+  </si>
+  <si>
+    <t>Separate defect metrics: store defective products separately from defect instances</t>
+  </si>
+  <si>
+    <t>Store defective products separately from defect instances.</t>
+  </si>
+  <si>
+    <t>Fast recipe statistics: change /recipes to read daily summary rows</t>
+  </si>
+  <si>
+    <t>Change /recipes to read daily summary rows.</t>
+  </si>
+  <si>
+    <t>Statistics migration verification: compare backfilled summary against source records</t>
+  </si>
+  <si>
+    <t>Compare backfilled summary against source records.</t>
+  </si>
+  <si>
+    <t>Nightly statistics reconciliation: periodically rebuild/check summary values</t>
+  </si>
+  <si>
+    <t>Periodically rebuild/check summary values.</t>
+  </si>
+  <si>
+    <t>Rebuild Statistics admin action: add administrator command to reconstruct summary rows</t>
+  </si>
+  <si>
+    <t>Add administrator command to reconstruct summary rows.</t>
+  </si>
+  <si>
+    <t>AI preview retention: add maximum age/size cleanup for AI images</t>
+  </si>
+  <si>
+    <t>Add maximum age/size cleanup for AI images.</t>
+  </si>
+  <si>
+    <t>Obsidian activity documentation: maintain architecture, installation and operating notes</t>
+  </si>
+  <si>
+    <t>Maintain architecture, installation and operating notes.</t>
   </si>
 </sst>
 </file>
@@ -5320,7 +5767,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1077"/>
+  <dimension ref="A1:N1151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -21715,6 +22162,2137 @@
       </c>
       <c r="M1077" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1078">
+        <v>547</v>
+      </c>
+      <c r="B1078" s="3" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C1078" s="3" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D1078" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1078" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1078" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1078">
+        <v>6</v>
+      </c>
+      <c r="J1078" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1078" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1079">
+        <v>548</v>
+      </c>
+      <c r="B1079" s="3" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C1079" s="3" t="s">
+        <v>1138</v>
+      </c>
+      <c r="D1079" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1079" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1079" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1079">
+        <v>8</v>
+      </c>
+      <c r="J1079" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1079" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1080">
+        <v>549</v>
+      </c>
+      <c r="B1080" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C1080" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="D1080" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1080" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1080" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1080">
+        <v>4</v>
+      </c>
+      <c r="J1080" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1080" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1081">
+        <v>550</v>
+      </c>
+      <c r="B1081" s="3" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C1081" s="3" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D1081" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1081" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1081" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1081">
+        <v>8</v>
+      </c>
+      <c r="J1081" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1081" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1082">
+        <v>551</v>
+      </c>
+      <c r="B1082" s="3" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C1082" s="3" t="s">
+        <v>1144</v>
+      </c>
+      <c r="D1082" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1082" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1082" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1082">
+        <v>8</v>
+      </c>
+      <c r="J1082" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1082" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1083">
+        <v>552</v>
+      </c>
+      <c r="B1083" s="3" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C1083" s="3" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D1083" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1083" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1083" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1083">
+        <v>4</v>
+      </c>
+      <c r="J1083" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1083" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1084">
+        <v>553</v>
+      </c>
+      <c r="B1084" s="3" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C1084" s="3" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D1084" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1084" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1084" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1084">
+        <v>3</v>
+      </c>
+      <c r="J1084" s="42">
+        <v>46262</v>
+      </c>
+      <c r="M1084" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1085">
+        <v>554</v>
+      </c>
+      <c r="B1085" s="3" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C1085" s="3" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D1085" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1085" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1085" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1085">
+        <v>4</v>
+      </c>
+      <c r="J1085" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1085" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1086">
+        <v>555</v>
+      </c>
+      <c r="B1086" s="3" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C1086" s="3" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D1086" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1086" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1086" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1086">
+        <v>4</v>
+      </c>
+      <c r="J1086" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1086" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1087">
+        <v>556</v>
+      </c>
+      <c r="B1087" s="3" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C1087" s="3" t="s">
+        <v>1154</v>
+      </c>
+      <c r="D1087" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1087" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1087" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1087">
+        <v>6</v>
+      </c>
+      <c r="J1087" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1087" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1088">
+        <v>557</v>
+      </c>
+      <c r="B1088" s="3" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C1088" s="3" t="s">
+        <v>1156</v>
+      </c>
+      <c r="D1088" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1088" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1088" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1088">
+        <v>10</v>
+      </c>
+      <c r="J1088" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1088" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1089">
+        <v>558</v>
+      </c>
+      <c r="B1089" s="3" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C1089" s="3" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D1089" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1089" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1089">
+        <v>4</v>
+      </c>
+      <c r="J1089" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1089" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1090">
+        <v>559</v>
+      </c>
+      <c r="B1090" s="3" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C1090" s="3" t="s">
+        <v>1160</v>
+      </c>
+      <c r="D1090" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1090" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1090" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1090">
+        <v>6</v>
+      </c>
+      <c r="J1090" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1090" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1091">
+        <v>560</v>
+      </c>
+      <c r="B1091" s="3" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C1091" s="3" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D1091" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1091" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1091" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1091">
+        <v>8</v>
+      </c>
+      <c r="J1091" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1091" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1092">
+        <v>561</v>
+      </c>
+      <c r="B1092" s="3" t="s">
+        <v>1163</v>
+      </c>
+      <c r="C1092" s="3" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D1092" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1092" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1092" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1092">
+        <v>8</v>
+      </c>
+      <c r="J1092" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1092" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1093">
+        <v>562</v>
+      </c>
+      <c r="B1093" s="3" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C1093" s="3" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D1093" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1093" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1093" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1093">
+        <v>2</v>
+      </c>
+      <c r="J1093" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1093" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1094">
+        <v>563</v>
+      </c>
+      <c r="B1094" s="3" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C1094" s="3" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D1094" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1094" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1094" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1094">
+        <v>16</v>
+      </c>
+      <c r="J1094" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1094" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1095">
+        <v>564</v>
+      </c>
+      <c r="B1095" s="3" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C1095" s="3" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D1095" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1095" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1095" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1095">
+        <v>6</v>
+      </c>
+      <c r="J1095" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1095" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1096">
+        <v>565</v>
+      </c>
+      <c r="B1096" s="3" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C1096" s="3" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D1096" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1096" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1096" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1096">
+        <v>3</v>
+      </c>
+      <c r="J1096" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1096" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1097">
+        <v>566</v>
+      </c>
+      <c r="B1097" s="3" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C1097" s="3" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D1097" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1097" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1097" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1097">
+        <v>4</v>
+      </c>
+      <c r="J1097" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1097" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1098">
+        <v>567</v>
+      </c>
+      <c r="B1098" s="3" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C1098" s="3" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D1098" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1098" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1098" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1098">
+        <v>2</v>
+      </c>
+      <c r="J1098" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1098" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1099">
+        <v>568</v>
+      </c>
+      <c r="B1099" s="3" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C1099" s="3" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D1099" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1099" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1099" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1099">
+        <v>2</v>
+      </c>
+      <c r="J1099" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1099" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1100">
+        <v>569</v>
+      </c>
+      <c r="B1100" s="3" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C1100" s="3" t="s">
+        <v>1180</v>
+      </c>
+      <c r="D1100" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1100" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1100" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1100">
+        <v>2</v>
+      </c>
+      <c r="J1100" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1100" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1101">
+        <v>570</v>
+      </c>
+      <c r="B1101" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C1101" s="3" t="s">
+        <v>1182</v>
+      </c>
+      <c r="D1101" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1101" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1101" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1101">
+        <v>5</v>
+      </c>
+      <c r="J1101" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1101" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1102">
+        <v>571</v>
+      </c>
+      <c r="B1102" s="3" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C1102" s="3" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D1102" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1102" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1102" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1102">
+        <v>4</v>
+      </c>
+      <c r="J1102" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1102" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1103">
+        <v>572</v>
+      </c>
+      <c r="B1103" s="3" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C1103" s="3" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D1103" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1103" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1103" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1103">
+        <v>5</v>
+      </c>
+      <c r="J1103" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1103" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1104">
+        <v>573</v>
+      </c>
+      <c r="B1104" s="3" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C1104" s="3" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D1104" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1104" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1104" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1104">
+        <v>3</v>
+      </c>
+      <c r="J1104" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1104" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1105">
+        <v>574</v>
+      </c>
+      <c r="B1105" s="3" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C1105" s="3" t="s">
+        <v>1190</v>
+      </c>
+      <c r="D1105" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1105" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1105" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1105">
+        <v>8</v>
+      </c>
+      <c r="J1105" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1105" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1106">
+        <v>575</v>
+      </c>
+      <c r="B1106" s="3" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C1106" s="3" t="s">
+        <v>1192</v>
+      </c>
+      <c r="D1106" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1106" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1106" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1106">
+        <v>6</v>
+      </c>
+      <c r="J1106" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1106" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1107">
+        <v>576</v>
+      </c>
+      <c r="B1107" s="3" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C1107" s="3" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D1107" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1107" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1107" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1107">
+        <v>3</v>
+      </c>
+      <c r="J1107" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1107" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1108">
+        <v>577</v>
+      </c>
+      <c r="B1108" s="3" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C1108" s="3" t="s">
+        <v>1196</v>
+      </c>
+      <c r="D1108" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1108" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1108" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1108">
+        <v>6</v>
+      </c>
+      <c r="J1108" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1108" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1109">
+        <v>578</v>
+      </c>
+      <c r="B1109" s="3" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C1109" s="3" t="s">
+        <v>1198</v>
+      </c>
+      <c r="D1109" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1109" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1109" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1109">
+        <v>4</v>
+      </c>
+      <c r="J1109" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1109" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1110">
+        <v>579</v>
+      </c>
+      <c r="B1110" s="3" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C1110" s="3" t="s">
+        <v>1200</v>
+      </c>
+      <c r="D1110" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1110" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1110" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1110">
+        <v>2</v>
+      </c>
+      <c r="J1110" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1110" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1111">
+        <v>580</v>
+      </c>
+      <c r="B1111" s="3" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C1111" s="3" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D1111" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1111" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1111" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1111">
+        <v>10</v>
+      </c>
+      <c r="J1111" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1111" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1112">
+        <v>581</v>
+      </c>
+      <c r="B1112" s="3" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C1112" s="3" t="s">
+        <v>1204</v>
+      </c>
+      <c r="D1112" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1112" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1112" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1112">
+        <v>6</v>
+      </c>
+      <c r="J1112" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1112" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1113">
+        <v>582</v>
+      </c>
+      <c r="B1113" s="3" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C1113" s="3" t="s">
+        <v>1206</v>
+      </c>
+      <c r="D1113" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1113" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1113" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1113">
+        <v>3</v>
+      </c>
+      <c r="J1113" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1113" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1114">
+        <v>583</v>
+      </c>
+      <c r="B1114" s="3" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C1114" s="3" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D1114" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1114" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1114" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1114">
+        <v>6</v>
+      </c>
+      <c r="J1114" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1114" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1115">
+        <v>584</v>
+      </c>
+      <c r="B1115" s="3" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C1115" s="3" t="s">
+        <v>1210</v>
+      </c>
+      <c r="D1115" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1115" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1115">
+        <v>1</v>
+      </c>
+      <c r="J1115" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1115" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1116">
+        <v>585</v>
+      </c>
+      <c r="B1116" s="3" t="s">
+        <v>1211</v>
+      </c>
+      <c r="C1116" s="3" t="s">
+        <v>1212</v>
+      </c>
+      <c r="D1116" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1116" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1116">
+        <v>3</v>
+      </c>
+      <c r="J1116" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1116" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1117">
+        <v>586</v>
+      </c>
+      <c r="B1117" s="3" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C1117" s="3" t="s">
+        <v>1214</v>
+      </c>
+      <c r="D1117" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1117" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1117">
+        <v>1</v>
+      </c>
+      <c r="J1117" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1117" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1118">
+        <v>587</v>
+      </c>
+      <c r="B1118" s="3" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C1118" s="3" t="s">
+        <v>1216</v>
+      </c>
+      <c r="D1118" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1118" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1118">
+        <v>3</v>
+      </c>
+      <c r="J1118" s="42">
+        <v>46263</v>
+      </c>
+      <c r="M1118" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1119">
+        <v>588</v>
+      </c>
+      <c r="B1119" s="3" t="s">
+        <v>1217</v>
+      </c>
+      <c r="C1119" s="3" t="s">
+        <v>1218</v>
+      </c>
+      <c r="D1119" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1119" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1119">
+        <v>8</v>
+      </c>
+      <c r="J1119" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1119" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1120">
+        <v>589</v>
+      </c>
+      <c r="B1120" s="3" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C1120" s="3" t="s">
+        <v>1220</v>
+      </c>
+      <c r="D1120" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1120" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1120">
+        <v>5</v>
+      </c>
+      <c r="J1120" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1120" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1121">
+        <v>590</v>
+      </c>
+      <c r="B1121" s="3" t="s">
+        <v>1221</v>
+      </c>
+      <c r="C1121" s="3" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D1121" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1121" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1121">
+        <v>6</v>
+      </c>
+      <c r="J1121" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1121" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1122">
+        <v>591</v>
+      </c>
+      <c r="B1122" s="3" t="s">
+        <v>1223</v>
+      </c>
+      <c r="C1122" s="3" t="s">
+        <v>1224</v>
+      </c>
+      <c r="D1122" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1122" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1122">
+        <v>3</v>
+      </c>
+      <c r="J1122" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1122" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1123">
+        <v>592</v>
+      </c>
+      <c r="B1123" s="3" t="s">
+        <v>1225</v>
+      </c>
+      <c r="C1123" s="3" t="s">
+        <v>1226</v>
+      </c>
+      <c r="D1123" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1123" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1123">
+        <v>4</v>
+      </c>
+      <c r="J1123" s="42">
+        <v>46265</v>
+      </c>
+      <c r="M1123" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1124">
+        <v>593</v>
+      </c>
+      <c r="B1124" s="3" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1124" s="3" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D1124" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1124" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1124">
+        <v>6</v>
+      </c>
+      <c r="M1124" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1125">
+        <v>594</v>
+      </c>
+      <c r="B1125" s="3" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C1125" s="3" t="s">
+        <v>1230</v>
+      </c>
+      <c r="D1125" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1125" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1125">
+        <v>6</v>
+      </c>
+      <c r="M1125" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1126">
+        <v>595</v>
+      </c>
+      <c r="B1126" s="3" t="s">
+        <v>1231</v>
+      </c>
+      <c r="C1126" s="3" t="s">
+        <v>1232</v>
+      </c>
+      <c r="D1126" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1126" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1126" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1126">
+        <v>8</v>
+      </c>
+      <c r="J1126" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1126" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1127">
+        <v>596</v>
+      </c>
+      <c r="B1127" s="3" t="s">
+        <v>1233</v>
+      </c>
+      <c r="C1127" s="3" t="s">
+        <v>1234</v>
+      </c>
+      <c r="D1127" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1127" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1127" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1127">
+        <v>12</v>
+      </c>
+      <c r="J1127" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1127" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1128">
+        <v>597</v>
+      </c>
+      <c r="B1128" s="3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C1128" s="3" t="s">
+        <v>1236</v>
+      </c>
+      <c r="D1128" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1128" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1128" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1128">
+        <v>4</v>
+      </c>
+      <c r="J1128" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1128" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1129">
+        <v>598</v>
+      </c>
+      <c r="B1129" s="3" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C1129" s="3" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D1129" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1129" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1129">
+        <v>3</v>
+      </c>
+      <c r="J1129" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1129" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1130">
+        <v>599</v>
+      </c>
+      <c r="B1130" s="3" t="s">
+        <v>1239</v>
+      </c>
+      <c r="C1130" s="3" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D1130" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1130" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1130" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1130">
+        <v>4</v>
+      </c>
+      <c r="J1130" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1130" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1131">
+        <v>600</v>
+      </c>
+      <c r="B1131" s="3" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C1131" s="3" t="s">
+        <v>1242</v>
+      </c>
+      <c r="D1131" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1131" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1131" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1131">
+        <v>4</v>
+      </c>
+      <c r="J1131" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1131" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1132">
+        <v>601</v>
+      </c>
+      <c r="B1132" s="3" t="s">
+        <v>1243</v>
+      </c>
+      <c r="C1132" s="3" t="s">
+        <v>1244</v>
+      </c>
+      <c r="D1132" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1132" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1132" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1132">
+        <v>5</v>
+      </c>
+      <c r="J1132" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1132" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1133">
+        <v>602</v>
+      </c>
+      <c r="B1133" s="3" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C1133" s="3" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D1133" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1133" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1133" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1133">
+        <v>3</v>
+      </c>
+      <c r="J1133" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1133" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1134">
+        <v>603</v>
+      </c>
+      <c r="B1134" s="3" t="s">
+        <v>1247</v>
+      </c>
+      <c r="C1134" s="3" t="s">
+        <v>1248</v>
+      </c>
+      <c r="D1134" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1134" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1134">
+        <v>4</v>
+      </c>
+      <c r="J1134" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1134" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1135">
+        <v>604</v>
+      </c>
+      <c r="B1135" s="3" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C1135" s="3" t="s">
+        <v>1250</v>
+      </c>
+      <c r="D1135" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1135" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1135" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1135">
+        <v>3</v>
+      </c>
+      <c r="J1135" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1135" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1136">
+        <v>605</v>
+      </c>
+      <c r="B1136" s="3" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C1136" s="3" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D1136" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1136" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1136" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1136">
+        <v>2</v>
+      </c>
+      <c r="J1136" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1136" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1137">
+        <v>606</v>
+      </c>
+      <c r="B1137" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C1137" s="3" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D1137" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1137" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1137" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1137">
+        <v>3</v>
+      </c>
+      <c r="J1137" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1137" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1138">
+        <v>607</v>
+      </c>
+      <c r="B1138" s="3" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C1138" s="3" t="s">
+        <v>1256</v>
+      </c>
+      <c r="D1138" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1138" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1138" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1138">
+        <v>3</v>
+      </c>
+      <c r="J1138" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1138" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1139">
+        <v>608</v>
+      </c>
+      <c r="B1139" s="3" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C1139" s="3" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D1139" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1139" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1139" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1139">
+        <v>3</v>
+      </c>
+      <c r="J1139" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1139" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1140">
+        <v>609</v>
+      </c>
+      <c r="B1140" s="3" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C1140" s="3" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D1140" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1140" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1140" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1140">
+        <v>4</v>
+      </c>
+      <c r="J1140" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1140" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1141">
+        <v>610</v>
+      </c>
+      <c r="B1141" s="3" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C1141" s="3" t="s">
+        <v>1262</v>
+      </c>
+      <c r="D1141" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1141" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1141" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1141">
+        <v>2</v>
+      </c>
+      <c r="J1141" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1141" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1142">
+        <v>611</v>
+      </c>
+      <c r="B1142" s="3" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C1142" s="3" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D1142" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1142" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1142" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1142">
+        <v>8</v>
+      </c>
+      <c r="J1142" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1142" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1143">
+        <v>612</v>
+      </c>
+      <c r="B1143" s="3" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C1143" s="3" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D1143" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1143" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1143" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1143">
+        <v>4</v>
+      </c>
+      <c r="J1143" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1143" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1144">
+        <v>613</v>
+      </c>
+      <c r="B1144" s="3" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C1144" s="3" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D1144" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1144" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1144" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1144">
+        <v>6</v>
+      </c>
+      <c r="J1144" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1144" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1145">
+        <v>614</v>
+      </c>
+      <c r="B1145" s="3" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C1145" s="3" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D1145" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1145" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1145" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1145">
+        <v>3</v>
+      </c>
+      <c r="J1145" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1145" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1146">
+        <v>615</v>
+      </c>
+      <c r="B1146" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C1146" s="3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D1146" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1146" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1146" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1146">
+        <v>4</v>
+      </c>
+      <c r="J1146" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1146" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1147">
+        <v>616</v>
+      </c>
+      <c r="B1147" s="3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C1147" s="3" t="s">
+        <v>1274</v>
+      </c>
+      <c r="D1147" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1147" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1147" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1147">
+        <v>2</v>
+      </c>
+      <c r="J1147" s="42">
+        <v>46267</v>
+      </c>
+      <c r="M1147" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1148">
+        <v>617</v>
+      </c>
+      <c r="B1148" s="3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C1148" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="D1148" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1148" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1148" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1148">
+        <v>6</v>
+      </c>
+      <c r="M1148" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1149">
+        <v>618</v>
+      </c>
+      <c r="B1149" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C1149" s="3" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D1149" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1149" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1149" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1149">
+        <v>5</v>
+      </c>
+      <c r="M1149" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1150">
+        <v>619</v>
+      </c>
+      <c r="B1150" s="3" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C1150" s="3" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D1150" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1150" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1150" t="s">
+        <v>427</v>
+      </c>
+      <c r="H1150">
+        <v>6</v>
+      </c>
+      <c r="M1150" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1151">
+        <v>620</v>
+      </c>
+      <c r="B1151" s="3" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C1151" s="3" t="s">
+        <v>1282</v>
+      </c>
+      <c r="D1151" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1151" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1151" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1151">
+        <v>6</v>
+      </c>
+      <c r="J1151" s="42">
+        <v>46264</v>
+      </c>
+      <c r="M1151" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -21843,15 +24421,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -22106,6 +24675,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -22118,14 +24696,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -22144,6 +24714,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add 2 Katana bug tasks (#621-#622): ABI.Unity issues #1213-#1214
#621 - Safety/PLC Error: door-open emergency error not shown in Katana (Backlog, Critical)
#622 - Page freeze during phantom mode / calibration offsets page (In review, Medium)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016CmAfMJ97kwanzK1vWp6P5
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497D3D87-B10F-49BA-A317-4A6C351579D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1341DD-930C-4E48-BC5B-1829C0698E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 Instructions" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3565" uniqueCount="1283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3575" uniqueCount="1287">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -3886,6 +3886,18 @@
   </si>
   <si>
     <t>Maintain architecture, installation and operating notes.</t>
+  </si>
+  <si>
+    <t>Safety / PLC Error Handling: door-open emergency error not shown in Katana</t>
+  </si>
+  <si>
+    <t>I opened the door; PLC was in Emergency error, but Katana was not showing any error.</t>
+  </si>
+  <si>
+    <t>Page freeze during phantom mode and on entering calibration offsets page</t>
+  </si>
+  <si>
+    <t>Page froze while phantom mode was running. Got stuck again after going into calibration offsets page.</t>
   </si>
 </sst>
 </file>
@@ -5468,7 +5480,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="438" row="1">
+  <wetp:taskpane dockstate="right" visibility="1" width="350" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -5767,7 +5779,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1151"/>
+  <dimension ref="A1:N1153"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -24293,6 +24305,52 @@
       </c>
       <c r="M1151" t="s">
         <v>182</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1152">
+        <v>621</v>
+      </c>
+      <c r="B1152" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C1152" s="3" t="s">
+        <v>1284</v>
+      </c>
+      <c r="E1152" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1152" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H1152">
+        <v>4</v>
+      </c>
+      <c r="M1152" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1153">
+        <v>622</v>
+      </c>
+      <c r="B1153" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C1153" s="3" t="s">
+        <v>1286</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1153" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1153">
+        <v>4</v>
+      </c>
+      <c r="M1153" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -24421,6 +24479,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -24675,15 +24742,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -24696,6 +24754,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -24714,14 +24780,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Sync 2026-09-21: 37 Katana status updates (#307-#622)
28 tasks -> Done: #316 #320 #325 #336 #338 #364 #464 #524-#536 #538-#544 #622
7 tasks -> In review: #307 #344 #345 #346 #348 #349 #362
2 tasks -> On Hold: #461 #465
Added 16 missing Excel rows for tasks #307-#465

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1341DD-930C-4E48-BC5B-1829C0698E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A491DD92-D752-4C4A-A4B2-1631F12C4029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37620" yWindow="615" windowWidth="17280" windowHeight="9960" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 Instructions" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3575" uniqueCount="1287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3655" uniqueCount="1304">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -3898,6 +3898,57 @@
   </si>
   <si>
     <t>Page froze while phantom mode was running. Got stuck again after going into calibration offsets page.</t>
+  </si>
+  <si>
+    <t>Draw a right hand showing arrows for direction of travel and X, Y, Z axes.</t>
+  </si>
+  <si>
+    <t>Each robot should clearly display its state: starting, running, stuck in dip and clean, or stopped.</t>
+  </si>
+  <si>
+    <t>Standardize alarms and alerts across the UI.</t>
+  </si>
+  <si>
+    <t>Spell out abbreviated setting names in full (e.g. Approach H).</t>
+  </si>
+  <si>
+    <t>General UI/UX: Camera page - add Restart Cameras button</t>
+  </si>
+  <si>
+    <t>Camera page: add a Restart Cameras button.</t>
+  </si>
+  <si>
+    <t>Logs: remove all debug logs, show only alarms.</t>
+  </si>
+  <si>
+    <t>Add multi-line selection in Custom Cut Mode.</t>
+  </si>
+  <si>
+    <t>Custom Cut Mode is not touch-friendly; optimize for touch.</t>
+  </si>
+  <si>
+    <t>Custom Cut Mode: Lock/hide normal parameters when enabled</t>
+  </si>
+  <si>
+    <t>When enabled, all normal parameters should be locked/hidden, and the current recipe should indicate custom cut.</t>
+  </si>
+  <si>
+    <t>Reorganize and rename settings menu items.</t>
+  </si>
+  <si>
+    <t>Remove FGF from everywhere.</t>
+  </si>
+  <si>
+    <t>Robot assignment alignment is off in the home preview.</t>
+  </si>
+  <si>
+    <t>Can't change the values on Blazor.</t>
+  </si>
+  <si>
+    <t>Auto-scale the cut preview so it always displays clearly.</t>
+  </si>
+  <si>
+    <t>Phantom images: allow users to turn on saving of phantom images.</t>
   </si>
 </sst>
 </file>
@@ -5779,7 +5830,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N1153"/>
+  <dimension ref="A1:N1169"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
@@ -21595,7 +21646,7 @@
         <v>1087</v>
       </c>
       <c r="E1055" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1055" t="s">
         <v>431</v>
@@ -21621,7 +21672,7 @@
         <v>1091</v>
       </c>
       <c r="E1056" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1056" t="s">
         <v>431</v>
@@ -21647,7 +21698,7 @@
         <v>1092</v>
       </c>
       <c r="E1057" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1057" t="s">
         <v>431</v>
@@ -21673,7 +21724,7 @@
         <v>1095</v>
       </c>
       <c r="E1058" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1058" t="s">
         <v>431</v>
@@ -21699,7 +21750,7 @@
         <v>1096</v>
       </c>
       <c r="E1059" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1059" t="s">
         <v>431</v>
@@ -21725,7 +21776,7 @@
         <v>1098</v>
       </c>
       <c r="E1060" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1060" t="s">
         <v>431</v>
@@ -21751,7 +21802,7 @@
         <v>1100</v>
       </c>
       <c r="E1061" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1061" t="s">
         <v>431</v>
@@ -21777,7 +21828,7 @@
         <v>1103</v>
       </c>
       <c r="E1062" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1062" t="s">
         <v>431</v>
@@ -21803,7 +21854,7 @@
         <v>1104</v>
       </c>
       <c r="E1063" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1063" t="s">
         <v>431</v>
@@ -21829,7 +21880,7 @@
         <v>1106</v>
       </c>
       <c r="E1064" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1064" t="s">
         <v>431</v>
@@ -21855,7 +21906,7 @@
         <v>1107</v>
       </c>
       <c r="E1065" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1065" t="s">
         <v>431</v>
@@ -21881,7 +21932,7 @@
         <v>1109</v>
       </c>
       <c r="E1066" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1066" t="s">
         <v>431</v>
@@ -21907,7 +21958,7 @@
         <v>1110</v>
       </c>
       <c r="E1067" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1067" t="s">
         <v>431</v>
@@ -21959,7 +22010,7 @@
         <v>1115</v>
       </c>
       <c r="E1069" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1069" t="s">
         <v>431</v>
@@ -21985,7 +22036,7 @@
         <v>1118</v>
       </c>
       <c r="E1070" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1070" t="s">
         <v>431</v>
@@ -22011,7 +22062,7 @@
         <v>1120</v>
       </c>
       <c r="E1071" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1071" t="s">
         <v>431</v>
@@ -22037,7 +22088,7 @@
         <v>1122</v>
       </c>
       <c r="E1072" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1072" t="s">
         <v>431</v>
@@ -22063,7 +22114,7 @@
         <v>1124</v>
       </c>
       <c r="E1073" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1073" t="s">
         <v>431</v>
@@ -22089,7 +22140,7 @@
         <v>1125</v>
       </c>
       <c r="E1074" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1074" t="s">
         <v>431</v>
@@ -22115,7 +22166,7 @@
         <v>1127</v>
       </c>
       <c r="E1075" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1075" t="s">
         <v>431</v>
@@ -24341,7 +24392,7 @@
         <v>1286</v>
       </c>
       <c r="E1153" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="F1153" t="s">
         <v>431</v>
@@ -24350,6 +24401,338 @@
         <v>4</v>
       </c>
       <c r="M1153" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1154">
+        <v>307</v>
+      </c>
+      <c r="B1154" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="C1154" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="E1154" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1154" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1154" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1155">
+        <v>316</v>
+      </c>
+      <c r="B1155" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="C1155" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="E1155" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1155" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1155" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1156">
+        <v>320</v>
+      </c>
+      <c r="B1156" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="C1156" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="E1156" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1156" t="s">
+        <v>428</v>
+      </c>
+      <c r="M1156" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1157">
+        <v>325</v>
+      </c>
+      <c r="B1157" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="C1157" s="3" t="s">
+        <v>1290</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1157" t="s">
+        <v>428</v>
+      </c>
+      <c r="M1157" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1158">
+        <v>336</v>
+      </c>
+      <c r="B1158" s="3" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C1158" s="3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="E1158" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1158" t="s">
+        <v>428</v>
+      </c>
+      <c r="M1158" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1159">
+        <v>338</v>
+      </c>
+      <c r="B1159" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C1159" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E1159" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1159" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1159">
+        <v>2</v>
+      </c>
+      <c r="M1159" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1160">
+        <v>344</v>
+      </c>
+      <c r="B1160" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1160" s="3" t="s">
+        <v>1294</v>
+      </c>
+      <c r="E1160" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1160" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1160" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1161">
+        <v>345</v>
+      </c>
+      <c r="B1161" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="C1161" s="3" t="s">
+        <v>1295</v>
+      </c>
+      <c r="E1161" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1161" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1161" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1162">
+        <v>346</v>
+      </c>
+      <c r="B1162" s="3" t="s">
+        <v>1296</v>
+      </c>
+      <c r="C1162" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="E1162" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1162" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1162" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1163">
+        <v>348</v>
+      </c>
+      <c r="B1163" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="C1163" s="3" t="s">
+        <v>1298</v>
+      </c>
+      <c r="E1163" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1163" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1163" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1164">
+        <v>349</v>
+      </c>
+      <c r="B1164" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="C1164" s="3" t="s">
+        <v>1299</v>
+      </c>
+      <c r="E1164" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1164" t="s">
+        <v>1136</v>
+      </c>
+      <c r="M1164" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1165">
+        <v>362</v>
+      </c>
+      <c r="B1165" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C1165" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="E1165" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1165" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1165">
+        <v>3</v>
+      </c>
+      <c r="M1165" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1166">
+        <v>364</v>
+      </c>
+      <c r="B1166" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="C1166" s="3" t="s">
+        <v>1300</v>
+      </c>
+      <c r="E1166" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1166" t="s">
+        <v>431</v>
+      </c>
+      <c r="M1166" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1167">
+        <v>461</v>
+      </c>
+      <c r="B1167" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="C1167" s="3" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E1167" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F1167" t="s">
+        <v>428</v>
+      </c>
+      <c r="H1167">
+        <v>1</v>
+      </c>
+      <c r="M1167" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1168">
+        <v>464</v>
+      </c>
+      <c r="B1168" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="C1168" s="3" t="s">
+        <v>1302</v>
+      </c>
+      <c r="E1168" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1168" t="s">
+        <v>431</v>
+      </c>
+      <c r="H1168">
+        <v>3</v>
+      </c>
+      <c r="M1168" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1169">
+        <v>465</v>
+      </c>
+      <c r="B1169" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="C1169" s="3" t="s">
+        <v>1303</v>
+      </c>
+      <c r="E1169" t="s">
+        <v>1068</v>
+      </c>
+      <c r="F1169" t="s">
+        <v>428</v>
+      </c>
+      <c r="M1169" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync 2026-10-05: 2 status updates + priority/assignee fills for #628-#661
Status changes:
- #642 (Grey out save button when not allowed) Backlog -> Done
- #646 (Auto dip and clean to recipe) Backlog -> Done

Metadata fills for 34 tasks (#628-#661):
- Priority now set from spreadsheet (High/Medium/Low as confirmed)
- Assignee filled for tasks with known GitHub logins (dilinaabi, MauricioDuqueABI)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_time_sheet.xlsx
+++ b/project_time_sheet.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D1AB1E-C469-4E40-A1AA-4EFF035FF54C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B4AD7D-A954-4152-8836-CF0E9DDF5EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3900" uniqueCount="1346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3921" uniqueCount="1346">
   <si>
     <t xml:space="preserve">  Project Time Sheet — User Guide</t>
   </si>
@@ -24978,11 +24978,14 @@
       <c r="B1175" s="3" t="s">
         <v>1310</v>
       </c>
+      <c r="D1175" t="s">
+        <v>61</v>
+      </c>
       <c r="E1175" t="s">
         <v>1304</v>
       </c>
       <c r="F1175" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1175" t="s">
         <v>1088</v>
@@ -25022,7 +25025,7 @@
         <v>1304</v>
       </c>
       <c r="F1177" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="K1177" t="s">
         <v>1088</v>
@@ -25038,6 +25041,9 @@
       <c r="B1178" s="3" t="s">
         <v>1313</v>
       </c>
+      <c r="D1178" t="s">
+        <v>61</v>
+      </c>
       <c r="E1178" t="s">
         <v>1304</v>
       </c>
@@ -25058,11 +25064,14 @@
       <c r="B1179" s="3" t="s">
         <v>1314</v>
       </c>
+      <c r="D1179" t="s">
+        <v>61</v>
+      </c>
       <c r="E1179" t="s">
         <v>1304</v>
       </c>
       <c r="F1179" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1179" t="s">
         <v>1088</v>
@@ -25078,11 +25087,14 @@
       <c r="B1180" s="3" t="s">
         <v>1315</v>
       </c>
+      <c r="D1180" t="s">
+        <v>61</v>
+      </c>
       <c r="E1180" t="s">
         <v>1304</v>
       </c>
       <c r="F1180" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="K1180" t="s">
         <v>1088</v>
@@ -25102,7 +25114,7 @@
         <v>1304</v>
       </c>
       <c r="F1181" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1181" t="s">
         <v>1088</v>
@@ -25142,7 +25154,7 @@
         <v>1304</v>
       </c>
       <c r="F1183" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="K1183" t="s">
         <v>1088</v>
@@ -25178,11 +25190,14 @@
       <c r="B1185" s="3" t="s">
         <v>1320</v>
       </c>
+      <c r="D1185" t="s">
+        <v>61</v>
+      </c>
       <c r="E1185" t="s">
         <v>1304</v>
       </c>
       <c r="F1185" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1185" t="s">
         <v>1088</v>
@@ -25198,11 +25213,14 @@
       <c r="B1186" s="3" t="s">
         <v>1321</v>
       </c>
+      <c r="D1186" t="s">
+        <v>61</v>
+      </c>
       <c r="E1186" t="s">
         <v>1304</v>
       </c>
       <c r="F1186" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K1186" t="s">
         <v>1088</v>
@@ -25218,11 +25236,14 @@
       <c r="B1187" s="3" t="s">
         <v>1322</v>
       </c>
+      <c r="D1187" t="s">
+        <v>61</v>
+      </c>
       <c r="E1187" t="s">
         <v>1304</v>
       </c>
       <c r="F1187" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="K1187" t="s">
         <v>1088</v>
@@ -25258,8 +25279,11 @@
       <c r="B1189" s="3" t="s">
         <v>1324</v>
       </c>
+      <c r="D1189" t="s">
+        <v>61</v>
+      </c>
       <c r="E1189" t="s">
-        <v>1304</v>
+        <v>78</v>
       </c>
       <c r="F1189" t="s">
         <v>431</v>
@@ -25278,6 +25302,9 @@
       <c r="B1190" s="3" t="s">
         <v>1325</v>
       </c>
+      <c r="D1190" t="s">
+        <v>61</v>
+      </c>
       <c r="E1190" t="s">
         <v>1304</v>
       </c>
@@ -25318,6 +25345,9 @@
       <c r="B1192" s="3" t="s">
         <v>1327</v>
       </c>
+      <c r="D1192" t="s">
+        <v>61</v>
+      </c>
       <c r="E1192" t="s">
         <v>1304</v>
       </c>
@@ -25338,11 +25368,14 @@
       <c r="B1193" s="3" t="s">
         <v>1328</v>
       </c>
+      <c r="D1193" t="s">
+        <v>61</v>
+      </c>
       <c r="E1193" t="s">
-        <v>1304</v>
+        <v>78</v>
       </c>
       <c r="F1193" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K1193" t="s">
         <v>1088</v>
@@ -25362,7 +25395,7 @@
         <v>1304</v>
       </c>
       <c r="F1194" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1194" t="s">
         <v>1088</v>
@@ -25378,6 +25411,9 @@
       <c r="B1195" s="3" t="s">
         <v>1330</v>
       </c>
+      <c r="D1195" t="s">
+        <v>61</v>
+      </c>
       <c r="E1195" t="s">
         <v>1304</v>
       </c>
@@ -25402,7 +25438,7 @@
         <v>1304</v>
       </c>
       <c r="F1196" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="K1196" t="s">
         <v>1088</v>
@@ -25418,11 +25454,14 @@
       <c r="B1197" s="3" t="s">
         <v>1332</v>
       </c>
+      <c r="D1197" t="s">
+        <v>61</v>
+      </c>
       <c r="E1197" t="s">
         <v>1304</v>
       </c>
       <c r="F1197" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1197" t="s">
         <v>1088</v>
@@ -25438,11 +25477,14 @@
       <c r="B1198" s="3" t="s">
         <v>1333</v>
       </c>
+      <c r="D1198" t="s">
+        <v>61</v>
+      </c>
       <c r="E1198" t="s">
         <v>1304</v>
       </c>
       <c r="F1198" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K1198" t="s">
         <v>1088</v>
@@ -25458,11 +25500,14 @@
       <c r="B1199" s="3" t="s">
         <v>1334</v>
       </c>
+      <c r="D1199" t="s">
+        <v>61</v>
+      </c>
       <c r="E1199" t="s">
         <v>1304</v>
       </c>
       <c r="F1199" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="K1199" t="s">
         <v>1088</v>
@@ -25518,11 +25563,14 @@
       <c r="B1202" s="3" t="s">
         <v>1337</v>
       </c>
+      <c r="D1202" t="s">
+        <v>62</v>
+      </c>
       <c r="E1202" t="s">
         <v>1304</v>
       </c>
       <c r="F1202" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K1202" t="s">
         <v>1088</v>
@@ -25558,6 +25606,9 @@
       <c r="B1204" s="3" t="s">
         <v>1339</v>
       </c>
+      <c r="D1204" t="s">
+        <v>61</v>
+      </c>
       <c r="E1204" t="s">
         <v>1304</v>
       </c>
@@ -25578,11 +25629,14 @@
       <c r="B1205" s="3" t="s">
         <v>1340</v>
       </c>
+      <c r="D1205" t="s">
+        <v>61</v>
+      </c>
       <c r="E1205" t="s">
         <v>1304</v>
       </c>
       <c r="F1205" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K1205" t="s">
         <v>1088</v>
@@ -25598,6 +25652,9 @@
       <c r="B1206" s="3" t="s">
         <v>1341</v>
       </c>
+      <c r="D1206" t="s">
+        <v>61</v>
+      </c>
       <c r="E1206" t="s">
         <v>1304</v>
       </c>
@@ -25618,6 +25675,9 @@
       <c r="B1207" s="3" t="s">
         <v>1342</v>
       </c>
+      <c r="D1207" t="s">
+        <v>61</v>
+      </c>
       <c r="E1207" t="s">
         <v>1304</v>
       </c>
@@ -25637,6 +25697,9 @@
       </c>
       <c r="B1208" s="3" t="s">
         <v>1343</v>
+      </c>
+      <c r="D1208" t="s">
+        <v>61</v>
       </c>
       <c r="E1208" t="s">
         <v>1304</v>
@@ -25953,15 +26016,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100959716F11FB6F9409089B98D1C11D330" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bc55ac45923017d94ee4534da3224188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2e20d828-e3fd-41fd-921c-fbe0ff523ae8" xmlns:ns3="adfc7943-f9ee-4478-a01e-ebfcb6e54f53" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5bc17ad4f23ab8382a0bb5b03decca58" ns2:_="" ns3:_="">
     <xsd:import namespace="2e20d828-e3fd-41fd-921c-fbe0ff523ae8"/>
@@ -26216,6 +26270,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -26228,14 +26291,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CE6A3B7-F954-4629-B802-2205DECE6851}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -26254,6 +26309,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{737DCCA1-99B2-40A5-A4E9-9FBBAC380C60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{407A8743-A532-48E3-9004-715BF423F4DA}">
   <ds:schemaRefs>

</xml_diff>